<commit_message>
Project 05: real per-port UARTs, V2.89 node handling, product-wise validation
RCA fixes: Port 1 routed to USART1 (J1) instead of the bench shortcut over USART2, which
made an empty Port 1 look online; single probe per cycle for offline ports (V2.89);
GetLcrNode answers the live node without scanning; immediate re-sync on SetPortLcrNode /
ModifyLcrNode; SetPortLcrNode refuses the same node on both ports; PresetGross/PresetNet
take the meter node like Start/Stop (tester + Leo's source).

Validation (J1 empty, J2 -> LCR simulator): product_suite 173/173, tracker_suite 129/129,
tester happy_flow on Port 2 59/63 (4 = BOXSTATUS_NO_METER for the empty J1).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PandaBox_Command_Test_Results_V2901.xlsx
+++ b/docs/PandaBox_Command_Test_Results_V2901.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -485,7 +485,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PC pandabox-tester (BLE) -&gt; PandaBox (GD32F305, bench build) -&gt; RS232 Port 2 -&gt; USB-RS232 COM7 -&gt; LCR simulator (meter 1 LCR-II node 1, meter 2 LCR.iQ node 2)</t>
+          <t>PC pandabox-tester (BLE) -&gt; PandaBox (GD32F305, bench build) -&gt; RS232 Port 2 (J2) -&gt; USB-RS232 COM7 -&gt; LCR simulator (LCR-II node 1, LCR.iQ node 2). Port 1 (J1): nothing connected.</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>137/137 passed (tools/tracker_suite.py)</t>
+          <t>129/129 passed (tools/tracker_suite.py)</t>
         </is>
       </c>
     </row>
@@ -509,66 +509,78 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>63/63 OK (pandabox-tester runner, validator v1.86)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Tracker cases by result</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>59/63 OK with the stock sequence re-pointed to Port 2 (SetPortLcrNode 0 1); the 4 flags are BOXSTATUS_NO_METER = J1 empty, correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Product-wise suite</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>173/173 (tools/product_suite.py: box, Port 1 empty, LCR-II and LCR.iQ on J2, node change, presets, delivery, history, unplug)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>83</v>
-      </c>
+          <t>Tracker cases by result</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DIFFERS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>DIFFERS</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>39</v>
+      <c r="B13" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -746,7 +758,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>HisDataTime 1 -&gt; LxHisDataTime 1,1790376044,1790376063,</t>
+          <t>HisDataTime 1 -&gt; LxHisDataTime 1,1790405494,1790405513,</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -845,8 +857,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>BoxStorage 1 -&gt; LxBoxStorage 1,15,24640,
-BoxStorage 2 -&gt; LxBoxStorage 2,8,25088,</t>
+          <t>BoxStorage 1 -&gt; LxBoxStorage 1,15,24640,</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr"/>
@@ -945,8 +956,8 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>GetData 1,1 -&gt; LxGetDataTs 1,0,1,1790376044,0.7,60.0,5154.3,0.0,5153.6,0.0,0.0,S,0.0,E
-GetDataEcho 1,0,1 -&gt; LxGetDataTs 1,0,2,1790376045,1.7,60.0,5155.3,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>GetData 1,1 -&gt; LxGetDataTs 1,0,6,1790405494,0.7,60.0,5391.6,0.0,5390.8,0.0,0.0,S,0.0,E
+GetDataEcho 6,0,1 -&gt; LxGetDataTs 1,0,7,1790405495,1.7,60.0,5392.5,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1016,7 +1027,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>GetData 1 0 -&gt; LxGetData 1,1,254,1790376049,5.6,60.0,5159.3,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>GetData 1 0 -&gt; LxGetData 1,1,132,1790405499,5.7,60.0,5396.5,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1156,7 +1167,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>GetDataTs 1,1790376040,1790376077 -&gt; LxGetDataTs 1,1,1790376045,1.7,60.0,5155.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,2,1790376046,2.6,60.0,5156.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,3,1790376047,3.6,60.0,5157.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,4,1790376048,4.6,60.0,5158.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,5,1790376049,5.6,60.0,5159.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,6,1790376050,6.6,60.0,5160.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,7,1790376051,7.6,60.0,5161.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,8,1790376052,8.7,60.0,5162.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,9,1790376053,9.1,0.0,5162.7,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,10,1790376059,9.7,60.0,5163.4,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,11,1790376060,10.7,60.0,5164.4,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,12,1790376061,11.7,60.0,5165.4,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,13,1790376062,12.7,60.0,5166.4,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,14,1790376063,13.2,0.0,5166.9,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,</t>
+          <t>GetDataTs 1,1790405490,1790405526 -&gt; LxGetDataTs 1,1,1790405495,1.7,60.0,5392.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,2,1790405496,2.7,60.0,5393.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,3,1790405497,3.7,60.0,5394.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,4,1790405498,4.7,60.0,5395.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,5,1790405499,5.7,60.0,5396.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,6,1790405500,6.7,60.0,5397.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,7,1790405501,7.7,60.0,5398.6,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,8,1790405502,8.7,60.0,5399.6,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,9,1790405503,9.1,0.0,5399.9,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,10,1790405509,9.6,60.0,5400.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,11,1790405510,10.6,60.0,5401.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,12,1790405511,11.6,60.0,5402.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,13,1790405512,12.7,60.0,5403.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,14,1790405513,13.4,0.0,5404.2,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1293,10 +1304,14 @@
       <c r="F21" s="3" t="inlineStr">
         <is>
           <t>DeleteAll 1 -&gt; LxDeleteAll 0
-DeleteAll 2 -&gt; LxDeleteAll 0</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr"/>
+DeleteAll 2 -&gt; LxDeleteAll 1</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>node 2 not configured on any port</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1789,7 +1804,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>BoxStatus -&gt; LxBoxStatus 2,0,1,2,0.0,S,0.0,E,0,1</t>
+          <t>BoxStatus -&gt; LxBoxStatus 2,0,0,1,0.0,S,0.0,E,0,1</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr"/>
@@ -1995,7 +2010,7 @@
           <t>BoxReset -&gt; LxBoxReset 0
 reconnect after BoxReset -&gt; 
 BoxInfo -&gt; LxBoxInfo 2.4,250502,2.901,260925,860858062040217,LCR
-SetBoxTime 1790376197 -&gt; LxSetBoxTime 0</t>
+SetBoxTime 1790405610 -&gt; LxSetBoxTime 0</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -2100,7 +2115,7 @@
       <c r="F45" s="3" t="inlineStr">
         <is>
           <t>SetRs485 1 -&gt; LxSetRs485 0
-RdRegister -&gt; LxRdRegister 1,1</t>
+RdRegister -&gt; LxRdRegister 0,1</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2138,12 +2153,12 @@
       <c r="F46" s="3" t="inlineStr">
         <is>
           <t>SetRs485 0 -&gt; LxSetRs485 0
-RdRegister -&gt; LxRdRegister 1,1</t>
+RdRegister -&gt; LxRdRegister 0,1</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>back on RS232 -&gt; meters online</t>
+          <t>back on RS232 -&gt; meter online</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2225,7 @@
         <is>
           <t>Start 1 -&gt; LxStart 0
 Start 1 -&gt; LxStart 0
-GetData 1 0 -&gt; LxGetData 1,1,10,1790376061,11.7,60.0,5165.4,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+GetData 1 0 -&gt; LxGetData 1,1,145,1790405512,12.7,60.0,5403.5,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -2339,7 +2354,7 @@
       <c r="F52" s="3" t="inlineStr">
         <is>
           <t>Pause 1 -&gt; LxPause 0
-GetData 1 0 -&gt; LxGetData 1,1,4,1790376055,9.1,0.0,5162.7,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+GetData 1 0 -&gt; LxGetData 1,1,138,1790405505,9.1,0.0,5399.9,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -2447,8 +2462,8 @@
       <c r="F55" s="3" t="inlineStr">
         <is>
           <t>Stop 1 -&gt; LxStop 0
-GetData 1 0 -&gt; LxGetData 1,1,14,1790376065,13.2,0.0,5166.9,0.0,5153.6,0.0,0.0,S,0.0,E
-GetData 1 0 (final) -&gt; LxGetData 1,1,14,1790376065,13.2,0.0,5166.9,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+GetData 1 0 -&gt; LxGetData 1,1,148,1790405515,13.4,0.0,5404.2,0.0,5390.8,0.0,0.0,S,0.0,E
+GetData 1 0 (final) -&gt; LxGetData 1,1,148,1790405515,13.4,0.0,5404.2,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2650,10 +2665,15 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>RdPortLcrNode -&gt; LxRdPortLcrNode 1,2</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr"/>
+          <t>RdPortLcrNode -&gt; LxRdPortLcrNode 1,2
+RdRegister -&gt; LxRdRegister 0,1</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>J1 empty; the simulator's LCR.iQ answers node 2 on J2</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -2716,10 +2736,10 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>ModifyLcrNode 1,1,5 -&gt; LxModifyLcrNode 0
-RdPortLcrNode -&gt; LxRdPortLcrNode 5,2
-GetData 5 0 -&gt; LxGetData 5,1,222,1790376017,15.1,0.0,5153.6,0.0,5138.5,0.0,0.0,S,0.0,E
-ModifyLcrNode 1,5,1 -&gt; LxModifyLcrNode 0</t>
+          <t>ModifyLcrNode 2,1,5 -&gt; LxModifyLcrNode 0
+RdPortLcrNode -&gt; LxRdPortLcrNode 0,5
+GetData 5 0 -&gt; LxGetData 5,1,103,1790405471,14.1,0.0,5390.8,0.0,5376.7,0.0,0.0,S,0.0,E
+ModifyLcrNode 2,5,1 -&gt; LxModifyLcrNode 0</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -2756,7 +2776,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>ModifyLcrNode 1,99,5 -&gt; LxModifyLcrNode 1</t>
+          <t>ModifyLcrNode 2,99,5 -&gt; LxModifyLcrNode 1</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr"/>
@@ -3020,7 +3040,7 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>BoxTime -&gt; LxBoxTime 1790375974</t>
+          <t>BoxTime -&gt; LxBoxTime 1790405426</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr"/>
@@ -3086,7 +3106,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>RdRegister -&gt; LxRdRegister 1,1</t>
+          <t>RdRegister -&gt; LxRdRegister 0,1</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr"/>
@@ -3119,12 +3139,12 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>RdRegister -&gt; LxRdRegister 1,0</t>
+          <t>RdRegister -&gt; LxRdRegister 0,0</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>port 2 empty -&gt; not registered</t>
+          <t>J1 empty, port 2 unassigned</t>
         </is>
       </c>
     </row>
@@ -3156,13 +3176,13 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>SwitchState 1 -&gt; LxSwitchState 1,Stop
-SwitchState 1 -&gt; LxSwitchState 1,Run</t>
+          <t>SwitchState 1 -&gt; LxSwitchState 1,Error
+SwitchState 2 -&gt; LxSwitchState 1,Run</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>delivery open</t>
+          <t>J1 empty; delivery open</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3214,7 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>SwitchState 2 -&gt; LxSwitchState 2,Stop</t>
+          <t>SwitchState 2 -&gt; LxSwitchState 1,Stop</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr"/>
@@ -3260,10 +3280,15 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>GetLcrNode 1,1,10 -&gt; LxFindLcrNode 1,1,</t>
-        </is>
-      </c>
-      <c r="G79" s="3" t="inlineStr"/>
+          <t>GetLcrNode 1,1,10 -&gt; LxFindLcrNode 0
+GetLcrNode 2,1,10 -&gt; LxFindLcrNode 2,1</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>J1 empty: scan finds nothing; J2 meter online -&gt; its node</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -3392,7 +3417,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>RdDiagnostics 1 -&gt; LxRdDiagnostics 0,1,0,26</t>
+          <t>RdDiagnostics 1 -&gt; LxRdDiagnostics 0,1,0,0</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr"/>
@@ -3525,11 +3550,15 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>RdMtrSetting 1 -&gt; LxRdMtrSetting 1,1,180,no,clear
-RdMtrSetting 2 -&gt; LxRdMtrSetting 2,2,180,no,clear</t>
-        </is>
-      </c>
-      <c r="G87" s="3" t="inlineStr"/>
+          <t>RdMtrSetting 1 -&gt; LxRdMtrSetting 1,Error
+RdMtrSetting 2 -&gt; LxRdMtrSetting 2,1,180,no,clear</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>J1 empty</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
@@ -3784,26 +3813,15 @@
           <t>1. Once the Panda Box is successfully connected to the app, for a dual-meter configuration, the Panda Box shall set the respective meter nodes for each port as provided by the app. It shall then reset both connected meters and fetch the totalizer value from each meter. 2. The fetched gallons/totalizer value for both meters shall match the corresponding totalizer value displayed on each meter.</t>
         </is>
       </c>
-      <c r="E96" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F96" s="3" t="inlineStr">
-        <is>
-          <t>Start 1 -&gt; LxStart 0
-Start 2 -&gt; LxStart 0
-GetData 1 0 -&gt; LxGetData 1,1,39,1790376090,4.6,60.0,5176.6,0.0,5171.9,0.0,0.0,S,0.0,E
-GetData 2 0 -&gt; LxGetData 2,1,36,1790376091,3.3,45.0,49295.4,0.0,49292.0,0.0,0.0,S,0.0,E
-Stop 1 -&gt; LxStop 0
-Stop 2 -&gt; LxStop 0
-GetData 1 0 -&gt; LxGetData 1,1,44,1790376095,7.0,0.0,5178.9,0.0,5171.9,0.0,0.0,S,0.0,E
-GetData 2 0 -&gt; LxGetData 2,1,41,1790376096,4.6,0.0,49296.6,0.0,49292.0,0.0,0.0,S,0.0,E</t>
-        </is>
-      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr"/>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>meter 1 flowing; meter 1 stopped; meter 2 flowing (independent); meter 2 stopped</t>
+          <t>Double meter needs a second meter on Port 1 (J1); the bench has one USB-RS232 adapter, on J2. Both products were validated one at a time on J2 (tools/product_suite.py)</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3848,11 @@
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr"/>
-      <c r="G97" s="3" t="inlineStr"/>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>Double meter wired crosswise needs two adapters (wrong-node handling checked in product_suite.py)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -3857,7 +3879,7 @@
       <c r="F98" s="3" t="inlineStr"/>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>One adapter carries both meters, so one meter cannot be unplugged alone; offline/online handling verified in PB-106</t>
+          <t>Only J2 is wired; a J1 with no meter is reported offline while J2 keeps working (PORT1 section of product_suite.py); unplug/replug verified in PB-106</t>
         </is>
       </c>
     </row>
@@ -3914,8 +3936,8 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>GetData 1 0 -&gt; LxGetData 1,1,0,1790376051,7.6,60.0,5161.3,0.0,5153.6,0.0,0.0,S,0.0,E
-GetData 1 0 x2 -&gt; LxGetData 1,1,254,1790376049,5.6,60.0,5159.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetData 1,1,0,1790376051,7.6,60.0,5161.3,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>GetData 1 0 -&gt; LxGetData 1,1,134,1790405501,7.7,60.0,5398.6,0.0,5390.8,0.0,0.0,S,0.0,E
+GetData 1 0 x2 -&gt; LxGetData 1,1,132,1790405499,5.7,60.0,5396.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetData 1,1,134,1790405501,7.7,60.0,5398.6,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
@@ -3977,7 +3999,7 @@
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>GetData 1 0 (paused) -&gt; LxGetData 1,1,6,1790376057,9.1,0.0,5162.7,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>GetData 1 0 (paused) -&gt; LxGetData 1,1,140,1790405507,9.1,0.0,5399.9,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
@@ -4130,15 +4152,15 @@
 RdRegister -&gt; LxRdRegister 0,0
 GetData 1 0 -&gt; LxGetData Error,
 Stop 1 -&gt; LxStop 1
-BoxStatus -&gt; LxBoxStatus 2,0,1,2,0.0,S,0.0,E,0,1
-RdRegister -&gt; LxRdRegister 1,1
-GetData 1 0 -&gt; LxGetData 1,1,52,1790376111,13.5,60.0,5192.5,0.0,5178.9,0.0,0.0,S,0.0,E
+BoxStatus -&gt; LxBoxStatus 2,0,0,1,0.0,S,0.0,E,0,1
+RdRegister -&gt; LxRdRegister 0,1
+GetData 1 0 -&gt; LxGetData 1,1,173,1790405548,13.5,60.0,5422.7,0.0,5409.2,0.0,0.0,S,0.0,E
 Stop 1 -&gt; LxStop 0</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>both meters offline; box still answers the app; command not delivered; delivery kept running on the meter while unplugged; meters back online after reconnect; no live data from an offline meter</t>
+          <t>box still answers the app; command not delivered; delivery kept running on the meter while unplugged; meter back online after reconnect; meter offline; no live data from an offline meter</t>
         </is>
       </c>
     </row>
@@ -4197,7 +4219,7 @@
         <is>
           <t>PresetGross 1,5.0 -&gt; LxPresetGross 0
 Start 1 -&gt; LxStart 0
-GetData 1 0 -&gt; LxGetData 1,1,31,1790376082,5.0,0.0,5171.9,0.0,5166.9,0.0,0.0,S,0.0,E</t>
+GetData 1 0 -&gt; LxGetData 1,1,165,1790405532,5.0,0.0,5409.2,0.0,5404.2,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
@@ -4826,7 +4848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H138"/>
+  <dimension ref="A1:H130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4892,7 +4914,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SetBoxTime 1790375964</t>
+          <t>SetBoxTime 1790405417</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4908,7 +4930,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>542.6</v>
+        <v>685.3</v>
       </c>
     </row>
     <row r="3">
@@ -4938,7 +4960,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>624.6</v>
+        <v>541</v>
       </c>
     </row>
     <row r="4">
@@ -4968,7 +4990,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>541.7</v>
+        <v>536</v>
       </c>
     </row>
     <row r="5">
@@ -4982,7 +5004,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SetPortLcrNode 1,2</t>
+          <t>SetPortLcrNode 0,1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4998,7 +5020,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>542.2</v>
+        <v>555.3</v>
       </c>
     </row>
     <row r="6">
@@ -5028,7 +5050,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>563.7</v>
+        <v>637.2</v>
       </c>
     </row>
     <row r="7">
@@ -5047,7 +5069,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LxStop 0</t>
+          <t>LxStop 1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5058,7 +5080,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>844.1</v>
+        <v>540.6</v>
       </c>
     </row>
     <row r="8">
@@ -5088,7 +5110,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>749.9</v>
+        <v>584</v>
       </c>
     </row>
     <row r="9">
@@ -5097,17 +5119,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SETUP</t>
+          <t>PB-035</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PresetGross 2,0</t>
+          <t>BoxStatus</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LxPresetGross 0</t>
+          <t>LxBoxStatus 2,0,0,1,0.0,S,0.0,E,0,1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -5118,7 +5140,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>571.8</v>
+        <v>705.2</v>
       </c>
     </row>
     <row r="10">
@@ -5127,17 +5149,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PB-035</t>
+          <t>PB-040</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BoxStatus</t>
+          <t>BoxInfo</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>LxBoxStatus 2,0,1,2,0.0,S,0.0,E,0,1</t>
+          <t>LxBoxInfo 2.4,250502,2.901,260925,860858062040217,LCR</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5148,7 +5170,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>539.1</v>
+        <v>542.3</v>
       </c>
     </row>
     <row r="11">
@@ -5157,17 +5179,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PB-040</t>
+          <t>PB-071</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BoxInfo</t>
+          <t>BoxTime</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LxBoxInfo 2.4,250502,2.901,260925,860858062040217,LCR</t>
+          <t>LxBoxTime 1790405426</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5175,10 +5197,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>box time should follow SetBoxTime</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>835.3</v>
+        <v>539.5</v>
       </c>
     </row>
     <row r="12">
@@ -5187,17 +5213,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PB-071</t>
+          <t>PB-042</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BoxTime</t>
+          <t>SetBoxTime 1748260000</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LxBoxTime 1790375974</t>
+          <t>LxSetBoxTime 0</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5205,14 +5231,10 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>box time should follow SetBoxTime</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>764.9</v>
+        <v>643.7</v>
       </c>
     </row>
     <row r="13">
@@ -5226,12 +5248,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SetBoxTime 1748260000</t>
+          <t>BoxTime</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>LxSetBoxTime 0</t>
+          <t>LxBoxTime 1748260000</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5239,10 +5261,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>time not applied</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>553.7</v>
+        <v>537.1</v>
       </c>
     </row>
     <row r="14">
@@ -5251,17 +5277,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PB-042</t>
+          <t>PB-043</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BoxTime</t>
+          <t>SetBoxTime -1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>LxBoxTime 1748260000</t>
+          <t>LxSetBoxTime 1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5269,14 +5295,10 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>time not applied</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>534.3</v>
+        <v>536.4</v>
       </c>
     </row>
     <row r="15">
@@ -5285,17 +5307,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PB-043</t>
+          <t>SETUP</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SetBoxTime -1</t>
+          <t>SetBoxTime 1790405429</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LxSetBoxTime 1</t>
+          <t>LxSetBoxTime 0</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5306,7 +5328,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>865</v>
+        <v>549.4</v>
       </c>
     </row>
     <row r="16">
@@ -5315,17 +5337,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SETUP</t>
+          <t>PB-022</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SetBoxTime 1790375977</t>
+          <t>RdBtName</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>LxSetBoxTime 0</t>
+          <t>LxRdBtName PandaBrain</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5336,7 +5358,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>542.2</v>
+        <v>535.9</v>
       </c>
     </row>
     <row r="17">
@@ -5345,17 +5367,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PB-022</t>
+          <t>PB-024</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>RdBtName</t>
+          <t>SetBtName AVeryLongNameOver16Bytes</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>LxRdBtName PandaBrain</t>
+          <t>LxSetBtName 1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5366,7 +5388,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>540.2</v>
+        <v>548.3</v>
       </c>
     </row>
     <row r="18">
@@ -5375,17 +5397,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PB-024</t>
+          <t>PB-025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SetBtName AVeryLongNameOver16Bytes</t>
+          <t>SetWifiName MyNetwork</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>LxSetBtName 1</t>
+          <t>LxSetWifiName 0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5396,7 +5418,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>677.3</v>
+        <v>546.4</v>
       </c>
     </row>
     <row r="19">
@@ -5405,17 +5427,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PB-025</t>
+          <t>PB-026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SetWifiName MyNetwork</t>
+          <t>SetWifiName AVeryLongNetworkNameHere</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LxSetWifiName 0</t>
+          <t>LxSetWifiName 1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5426,7 +5448,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>548.9</v>
+        <v>541.1</v>
       </c>
     </row>
     <row r="20">
@@ -5435,17 +5457,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PB-026</t>
+          <t>PB-027</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SetWifiName AVeryLongNetworkNameHere</t>
+          <t>SetWifiPwd mypassword</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LxSetWifiName 1</t>
+          <t>LxSetWifiPwd 0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5456,7 +5478,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>541.1</v>
+        <v>543.2</v>
       </c>
     </row>
     <row r="21">
@@ -5465,17 +5487,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PB-027</t>
+          <t>PB-028</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SetWifiPwd mypassword</t>
+          <t>SetWifiPwd averylongpasswordthatexceeds</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LxSetWifiPwd 0</t>
+          <t>LxSetWifiPwd 1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -5486,7 +5508,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>864.3</v>
+        <v>547.3</v>
       </c>
     </row>
     <row r="22">
@@ -5495,17 +5517,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PB-028</t>
+          <t>PB-029</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SetWifiPwd averylongpasswordthatexceeds</t>
+          <t>SetServerIp 13.205.61.50</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>LxSetWifiPwd 1</t>
+          <t>LxSetServerIp 0</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5516,7 +5538,7 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>764.6</v>
+        <v>547.5</v>
       </c>
     </row>
     <row r="23">
@@ -5525,17 +5547,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PB-029</t>
+          <t>PB-030</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SetServerIp 13.205.61.50</t>
+          <t>SetServerIp 999.9999.999.999</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>LxSetServerIp 0</t>
+          <t>LxSetServerIp 1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5546,7 +5568,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>541.2</v>
+        <v>546.8</v>
       </c>
     </row>
     <row r="24">
@@ -5555,17 +5577,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PB-030</t>
+          <t>PB-031</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SetServerIp 999.9999.999.999</t>
+          <t>SetServerPort 8181</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>LxSetServerIp 1</t>
+          <t>LxSetServerPort 0</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5576,7 +5598,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>543</v>
+        <v>546.6</v>
       </c>
     </row>
     <row r="25">
@@ -5585,17 +5607,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PB-031</t>
+          <t>PB-032</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SetServerPort 8181</t>
+          <t>SetServerPort 99999</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>LxSetServerPort 0</t>
+          <t>LxSetServerPort 1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -5606,7 +5628,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>872.4</v>
+        <v>728.5</v>
       </c>
     </row>
     <row r="26">
@@ -5615,17 +5637,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PB-032</t>
+          <t>PB-033</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SetServerPort 99999</t>
+          <t>SetApn jionet</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>LxSetServerPort 1</t>
+          <t>LxSetApn 0</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -5636,7 +5658,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>542.6</v>
+        <v>535.6</v>
       </c>
     </row>
     <row r="27">
@@ -5645,17 +5667,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PB-033</t>
+          <t>PB-034</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SetApn jionet</t>
+          <t>SetApn</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>LxSetApn 0</t>
+          <t>LxSetApn 1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -5666,7 +5688,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>539.8</v>
+        <v>540.7</v>
       </c>
     </row>
     <row r="28">
@@ -5675,17 +5697,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PB-034</t>
+          <t>PB-036</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SetApn</t>
+          <t>SetMode 2</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>LxSetApn 1</t>
+          <t>LxSetMode 0</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -5696,7 +5718,7 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>646.8</v>
+        <v>540.7</v>
       </c>
     </row>
     <row r="29">
@@ -5705,12 +5727,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PB-036</t>
+          <t>PB-037</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SetMode 2</t>
+          <t>SetMode 1</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -5726,7 +5748,7 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>534.3</v>
+        <v>540.8</v>
       </c>
     </row>
     <row r="30">
@@ -5740,12 +5762,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SetMode 1</t>
+          <t>GetData 1 0</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>LxSetMode 0</t>
+          <t>LxGetData Mode 1,</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5754,9 +5776,13 @@
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>bridge mode: meter data not served</t>
+        </is>
+      </c>
       <c r="H30" t="n">
-        <v>534</v>
+        <v>546.1</v>
       </c>
     </row>
     <row r="31">
@@ -5765,17 +5791,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PB-037</t>
+          <t>PB-038</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>SetMode 3</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>LxGetData Mode 1,</t>
+          <t>LxSetMode 0</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5784,13 +5810,9 @@
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>bridge mode: meter data not served</t>
-        </is>
-      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>897</v>
+        <v>541.3</v>
       </c>
     </row>
     <row r="32">
@@ -5799,17 +5821,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PB-038</t>
+          <t>PB-039</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SetMode 3</t>
+          <t>SetMode 5</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>LxSetMode 0</t>
+          <t>LxSetMode 1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -5820,7 +5842,7 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>764.3</v>
+        <v>535.4</v>
       </c>
     </row>
     <row r="33">
@@ -5829,17 +5851,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PB-039</t>
+          <t>SETUP</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SetMode 5</t>
+          <t>SetMode 2</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>LxSetMode 1</t>
+          <t>LxSetMode 0</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5850,7 +5872,7 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>535.7</v>
+        <v>539.6</v>
       </c>
     </row>
     <row r="34">
@@ -5859,17 +5881,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SETUP</t>
+          <t>PB-044</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SetMode 2</t>
+          <t>SetRs485 1</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LxSetMode 0</t>
+          <t>LxSetRs485 0</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5880,7 +5902,7 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>544.6</v>
+        <v>540.6</v>
       </c>
     </row>
     <row r="35">
@@ -5894,12 +5916,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SetRs485 1</t>
+          <t>RdRegister</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LxSetRs485 0</t>
+          <t>LxRdRegister 0,1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5908,9 +5930,13 @@
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>info: PE5 off / PE6 on is verified on the pins; this bench's RS232 chip still passes data</t>
+        </is>
+      </c>
       <c r="H35" t="n">
-        <v>901.4</v>
+        <v>790.3</v>
       </c>
     </row>
     <row r="36">
@@ -5919,17 +5945,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PB-044</t>
+          <t>PB-045</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>RdRegister</t>
+          <t>SetRs485 0</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LxRdRegister 1,1</t>
+          <t>LxSetRs485 0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -5938,13 +5964,9 @@
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>info: PE5 off / PE6 on is verified on the pins; this bench's RS232 chip still passes data</t>
-        </is>
-      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>609.4</v>
+        <v>538.8</v>
       </c>
     </row>
     <row r="37">
@@ -5958,12 +5980,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SetRs485 0</t>
+          <t>RdRegister</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>LxSetRs485 0</t>
+          <t>LxRdRegister 0,1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5972,9 +5994,13 @@
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>back on RS232 -&gt; meter online</t>
+        </is>
+      </c>
       <c r="H37" t="n">
-        <v>540.7</v>
+        <v>542</v>
       </c>
     </row>
     <row r="38">
@@ -5983,17 +6009,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PB-045</t>
+          <t>PB-046</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>RdRegister</t>
+          <t>SetRs485 2</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>LxRdRegister 1,1</t>
+          <t>LxSetRs485 1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -6002,13 +6028,9 @@
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>back on RS232 -&gt; meters online</t>
-        </is>
-      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>811.1</v>
+        <v>651.7</v>
       </c>
     </row>
     <row r="39">
@@ -6017,17 +6039,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PB-046</t>
+          <t>PB-057</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SetRs485 2</t>
+          <t>SetPortLcrNode 1,2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>LxSetRs485 1</t>
+          <t>LxSetPortLcrNode 0</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -6038,7 +6060,7 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>757.4</v>
+        <v>547.7</v>
       </c>
     </row>
     <row r="40">
@@ -6047,17 +6069,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PB-057</t>
+          <t>PB-060</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SetPortLcrNode 1,2</t>
+          <t>RdPortLcrNode</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>LxSetPortLcrNode 0</t>
+          <t>LxRdPortLcrNode 1,2</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -6068,7 +6090,7 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>541.9</v>
+        <v>658.9</v>
       </c>
     </row>
     <row r="41">
@@ -6082,12 +6104,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>RdPortLcrNode</t>
+          <t>RdRegister</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>LxRdPortLcrNode 1,2</t>
+          <t>LxRdRegister 0,1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -6096,9 +6118,13 @@
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>J1 empty; the simulator's LCR.iQ answers node 2 on J2</t>
+        </is>
+      </c>
       <c r="H41" t="n">
-        <v>535.8</v>
+        <v>541.9</v>
       </c>
     </row>
     <row r="42">
@@ -6128,7 +6154,7 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>885</v>
+        <v>546.9</v>
       </c>
     </row>
     <row r="43">
@@ -6158,7 +6184,7 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>536.6</v>
+        <v>537.9</v>
       </c>
     </row>
     <row r="44">
@@ -6177,7 +6203,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>LxRdRegister 1,0</t>
+          <t>LxRdRegister 0,0</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -6188,11 +6214,11 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>port 2 empty -&gt; not registered</t>
+          <t>J1 empty, port 2 unassigned</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>533.8</v>
+        <v>534.9</v>
       </c>
     </row>
     <row r="45">
@@ -6222,7 +6248,7 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>700.3</v>
+        <v>584.6</v>
       </c>
     </row>
     <row r="46">
@@ -6236,7 +6262,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SetPortLcrNode 1,2</t>
+          <t>SetPortLcrNode 0,1</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -6252,7 +6278,7 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>547.7</v>
+        <v>549.3</v>
       </c>
     </row>
     <row r="47">
@@ -6271,7 +6297,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>LxRdRegister 1,1</t>
+          <t>LxRdRegister 0,1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -6282,7 +6308,7 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>546.6</v>
+        <v>598.4</v>
       </c>
     </row>
     <row r="48">
@@ -6301,7 +6327,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>LxSwitchState 1,Stop</t>
+          <t>LxSwitchState 1,Error</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -6310,9 +6336,13 @@
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>J1 empty</t>
+        </is>
+      </c>
       <c r="H48" t="n">
-        <v>739.7</v>
+        <v>541.7</v>
       </c>
     </row>
     <row r="49">
@@ -6331,7 +6361,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>LxSwitchState 2,Stop</t>
+          <t>LxSwitchState 1,Stop</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -6342,7 +6372,7 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>539.7</v>
+        <v>614.8</v>
       </c>
     </row>
     <row r="50">
@@ -6372,7 +6402,7 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>534.4</v>
+        <v>541.6</v>
       </c>
     </row>
     <row r="51">
@@ -6391,7 +6421,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>LxFindLcrNode 1,1,</t>
+          <t>LxFindLcrNode 0</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -6400,9 +6430,13 @@
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>J1 empty: scan finds nothing</t>
+        </is>
+      </c>
       <c r="H51" t="n">
-        <v>909.5</v>
+        <v>1777.8</v>
       </c>
     </row>
     <row r="52">
@@ -6411,17 +6445,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PB-079</t>
+          <t>PB-078</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>GetLcrNode 1,200,10</t>
+          <t>GetLcrNode 2,1,10</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>LxFindLcrNode 0</t>
+          <t>LxFindLcrNode 2,1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -6430,9 +6464,13 @@
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>J2 meter online -&gt; its node</t>
+        </is>
+      </c>
       <c r="H52" t="n">
-        <v>735.3</v>
+        <v>539.8</v>
       </c>
     </row>
     <row r="53">
@@ -6441,12 +6479,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PB-080</t>
+          <t>PB-079</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>GetLcrNode 1,1,251</t>
+          <t>GetLcrNode 1,200,10</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6462,7 +6500,7 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>547.5</v>
+        <v>547.4</v>
       </c>
     </row>
     <row r="54">
@@ -6471,17 +6509,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PB-062</t>
+          <t>PB-080</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ModifyLcrNode 1,1,5</t>
+          <t>GetLcrNode 1,1,251</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>LxModifyLcrNode 0</t>
+          <t>LxFindLcrNode 0</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -6492,7 +6530,7 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>571.9</v>
+        <v>711.8</v>
       </c>
     </row>
     <row r="55">
@@ -6506,12 +6544,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RdPortLcrNode</t>
+          <t>ModifyLcrNode 2,1,5</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>LxRdPortLcrNode 5,2</t>
+          <t>LxModifyLcrNode 0</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6522,7 +6560,7 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>854.1</v>
+        <v>795.1</v>
       </c>
     </row>
     <row r="56">
@@ -6536,12 +6574,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>GetData 5 0</t>
+          <t>RdPortLcrNode</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>LxGetData 5,1,222,1790376017,15.1,0.0,5153.6,0.0,5138.5,0.0,0.0,S,0.0,E</t>
+          <t>LxRdPortLcrNode 0,5</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -6550,13 +6588,9 @@
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>meter answers on its new node 5</t>
-        </is>
-      </c>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>542.9</v>
+        <v>539.7</v>
       </c>
     </row>
     <row r="57">
@@ -6570,12 +6604,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ModifyLcrNode 1,5,1</t>
+          <t>GetData 5 0</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>LxModifyLcrNode 0</t>
+          <t>LxGetData 5,1,103,1790405471,14.1,0.0,5390.8,0.0,5376.7,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -6586,11 +6620,11 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>restore node 1</t>
+          <t>meter answers on its new node 5</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>564.6</v>
+        <v>656.2</v>
       </c>
     </row>
     <row r="58">
@@ -6599,17 +6633,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PB-063</t>
+          <t>PB-062</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ModifyLcrNode 1,99,5</t>
+          <t>ModifyLcrNode 2,5,1</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>LxModifyLcrNode 1</t>
+          <t>LxModifyLcrNode 0</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -6618,9 +6652,13 @@
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>restore node 1</t>
+        </is>
+      </c>
       <c r="H58" t="n">
-        <v>971.5</v>
+        <v>811.2</v>
       </c>
     </row>
     <row r="59">
@@ -6629,12 +6667,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PB-064</t>
+          <t>PB-063</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ModifyLcrNode 3,1,5</t>
+          <t>ModifyLcrNode 2,99,5</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -6650,7 +6688,7 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>868.2</v>
+        <v>665.2</v>
       </c>
     </row>
     <row r="60">
@@ -6659,17 +6697,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PB-086</t>
+          <t>PB-064</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>RdMtrSetting 1</t>
+          <t>ModifyLcrNode 3,1,5</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>LxRdMtrSetting 1,1,180,no,clear</t>
+          <t>LxModifyLcrNode 1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -6680,7 +6718,7 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>891.9</v>
+        <v>548.5</v>
       </c>
     </row>
     <row r="61">
@@ -6694,12 +6732,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>RdMtrSetting 2</t>
+          <t>RdMtrSetting 1</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>LxRdMtrSetting 2,2,180,no,clear</t>
+          <t>LxRdMtrSetting 1,Error</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -6708,9 +6746,13 @@
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>J1 empty</t>
+        </is>
+      </c>
       <c r="H61" t="n">
-        <v>983.8</v>
+        <v>540.2</v>
       </c>
     </row>
     <row r="62">
@@ -6719,17 +6761,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PB-087</t>
+          <t>PB-086</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>RdMtrSetting 3</t>
+          <t>RdMtrSetting 2</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>LxRdMtrSetting 3,Error</t>
+          <t>LxRdMtrSetting 2,1,180,no,clear</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -6740,7 +6782,7 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>857.6</v>
+        <v>683</v>
       </c>
     </row>
     <row r="63">
@@ -6749,17 +6791,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PB-082</t>
+          <t>PB-087</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>RdDiagnostics 1</t>
+          <t>RdMtrSetting 3</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>LxRdDiagnostics 0,1,0,26</t>
+          <t>LxRdMtrSetting 3,Error</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -6770,7 +6812,7 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>541.4</v>
+        <v>538.9</v>
       </c>
     </row>
     <row r="64">
@@ -6779,17 +6821,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PB-083</t>
+          <t>PB-082</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>RdDiagnostics 99</t>
+          <t>RdDiagnostics 1</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>LxRdDiagnostics 99,Error</t>
+          <t>LxRdDiagnostics 0,1,0,0</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -6800,7 +6842,7 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>540.6</v>
+        <v>534.4</v>
       </c>
     </row>
     <row r="65">
@@ -6809,17 +6851,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PB-081</t>
+          <t>PB-083</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>GetLastCmd</t>
+          <t>RdDiagnostics 99</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>LxGetLastCmd 1,0</t>
+          <t>LxRdDiagnostics 99,Error</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -6830,7 +6872,7 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>645.2</v>
+        <v>540.3</v>
       </c>
     </row>
     <row r="66">
@@ -6839,17 +6881,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PB-085</t>
+          <t>PB-081</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>GetLastMtrCmd 99</t>
+          <t>GetLastCmd</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>LxGetLastMtrCmd 99,None,1</t>
+          <t>LxGetLastCmd 1,0</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6860,7 +6902,7 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>536.4</v>
+        <v>548.6</v>
       </c>
     </row>
     <row r="67">
@@ -6869,17 +6911,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PB-020</t>
+          <t>PB-085</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>DeleteAll 1</t>
+          <t>GetLastMtrCmd 99</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>LxDeleteAll 0</t>
+          <t>LxGetLastMtrCmd 99,None,1</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6890,7 +6932,7 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>533.2</v>
+        <v>536.2</v>
       </c>
     </row>
     <row r="68">
@@ -6904,7 +6946,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>DeleteAll 2</t>
+          <t>DeleteAll 1</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -6920,7 +6962,7 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>888.2</v>
+        <v>539.1</v>
       </c>
     </row>
     <row r="69">
@@ -6929,12 +6971,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PB-021</t>
+          <t>PB-020</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>DeleteAll 99</t>
+          <t>DeleteAll 2</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -6948,9 +6990,13 @@
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>node 2 not configured on any port</t>
+        </is>
+      </c>
       <c r="H69" t="n">
-        <v>764.5</v>
+        <v>535.1</v>
       </c>
     </row>
     <row r="70">
@@ -6959,17 +7005,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PB-006</t>
+          <t>PB-021</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>HisDataTime 1</t>
+          <t>DeleteAll 99</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>LxHisDataTime 1,</t>
+          <t>LxDeleteAll 1</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6980,7 +7026,7 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>535.8</v>
+        <v>540.2</v>
       </c>
     </row>
     <row r="71">
@@ -6989,17 +7035,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PB-005</t>
+          <t>PB-006</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>HisDataTime 99</t>
+          <t>HisDataTime 1</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>LxHisDataTime 99,</t>
+          <t>LxHisDataTime 1,</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -7010,7 +7056,7 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>539.5</v>
+        <v>653.4</v>
       </c>
     </row>
     <row r="72">
@@ -7019,17 +7065,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PB-009</t>
+          <t>PB-005</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>BoxStorage 99</t>
+          <t>HisDataTime 99</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>LxBoxStorage 99,0,25600,</t>
+          <t>LxHisDataTime 99,</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -7040,7 +7086,7 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>889.6</v>
+        <v>541.5</v>
       </c>
     </row>
     <row r="73">
@@ -7049,17 +7095,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PB-013</t>
+          <t>PB-009</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>GetData 1,1</t>
+          <t>BoxStorage 99</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>LxGetDataTs 1,</t>
+          <t>LxBoxStorage 99,0,25600,</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -7068,13 +7114,9 @@
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>storage empty</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>540.6</v>
+        <v>541.2</v>
       </c>
     </row>
     <row r="74">
@@ -7083,17 +7125,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PB-015</t>
+          <t>PB-013</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>GetData 99,1</t>
+          <t>GetData 1,1</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>LxGetData Error,</t>
+          <t>LxGetDataTs 1,</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -7102,9 +7144,13 @@
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>storage empty</t>
+        </is>
+      </c>
       <c r="H74" t="n">
-        <v>540</v>
+        <v>644.3</v>
       </c>
     </row>
     <row r="75">
@@ -7113,17 +7159,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PB-017</t>
+          <t>PB-015</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>GetDataTs 1,1700000000,1700003600</t>
+          <t>GetData 99,1</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>LxGetDataTs 1,</t>
+          <t>LxGetData Error,</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -7134,7 +7180,7 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>661.2</v>
+        <v>534.8</v>
       </c>
     </row>
     <row r="76">
@@ -7143,12 +7189,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PB-018</t>
+          <t>PB-017</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>GetDataTs 1,1700003600,1700000000</t>
+          <t>GetDataTs 1,1700000000,1700003600</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7164,7 +7210,7 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>543.7</v>
+        <v>541.6</v>
       </c>
     </row>
     <row r="77">
@@ -7173,12 +7219,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PB-019</t>
+          <t>PB-018</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>GetDataTs 1,1700000000,1700000001</t>
+          <t>GetDataTs 1,1700003600,1700000000</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7194,7 +7240,7 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>548.3</v>
+        <v>549.5</v>
       </c>
     </row>
     <row r="78">
@@ -7203,17 +7249,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PB-065</t>
+          <t>PB-019</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>PresetGross 1,125.5</t>
+          <t>GetDataTs 1,1700000000,1700000001</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>LxPresetGross 0</t>
+          <t>LxGetDataTs 1,</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7224,7 +7270,7 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>894.8</v>
+        <v>548.9</v>
       </c>
     </row>
     <row r="79">
@@ -7233,17 +7279,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PB-066</t>
+          <t>PB-065</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>PresetGross 3,125.5</t>
+          <t>PresetGross 1,125.5</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>LxPresetGross 1</t>
+          <t>LxPresetGross 0</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7254,7 +7300,7 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>734</v>
+        <v>572.5</v>
       </c>
     </row>
     <row r="80">
@@ -7263,12 +7309,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PB-067</t>
+          <t>PB-066</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>PresetGross 1,-10.0</t>
+          <t>PresetGross 3,125.5</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7284,7 +7330,7 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>580.4</v>
+        <v>546.6</v>
       </c>
     </row>
     <row r="81">
@@ -7293,17 +7339,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PB-068</t>
+          <t>PB-067</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>PresetNet 1,125.5</t>
+          <t>PresetGross 1,-10.0</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>LxPresetNet 0</t>
+          <t>LxPresetGross 1</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7314,7 +7360,7 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>577.9</v>
+        <v>586.8</v>
       </c>
     </row>
     <row r="82">
@@ -7323,17 +7369,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PB-069</t>
+          <t>PB-068</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>PresetNet 3,125.5</t>
+          <t>PresetNet 1,125.5</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>LxPresetNet 1</t>
+          <t>LxPresetNet 0</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7344,7 +7390,7 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>796.5</v>
+        <v>577.8</v>
       </c>
     </row>
     <row r="83">
@@ -7353,12 +7399,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PB-070</t>
+          <t>PB-069</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>PresetNet 1,-10.0</t>
+          <t>PresetNet 3,125.5</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7374,7 +7420,7 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>574.6</v>
+        <v>541.2</v>
       </c>
     </row>
     <row r="84">
@@ -7383,17 +7429,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SETUP</t>
+          <t>PB-070</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>PresetGross 1,0</t>
+          <t>PresetNet 1,-10.0</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>LxPresetGross 0</t>
+          <t>LxPresetNet 1</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -7404,7 +7450,7 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>569.3</v>
+        <v>676.8</v>
       </c>
     </row>
     <row r="85">
@@ -7418,12 +7464,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>PresetNet 1,0</t>
+          <t>PresetGross 1,0</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>LxPresetNet 0</t>
+          <t>LxPresetGross 0</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -7434,7 +7480,7 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>641</v>
+        <v>571.9</v>
       </c>
     </row>
     <row r="86">
@@ -7443,17 +7489,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PB-052</t>
+          <t>SETUP</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Pause 1</t>
+          <t>PresetNet 1,0</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>LxPause 0</t>
+          <t>LxPresetNet 0</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -7462,13 +7508,9 @@
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>V2.89 + real LCR: Pause with no delivery open is accepted (rc 0, devSt 0x21 in the golden capture); the tracker's LxPause 1 is the V3.01 firmware guard</t>
-        </is>
-      </c>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>569.9</v>
+        <v>578.7</v>
       </c>
     </row>
     <row r="87">
@@ -7477,17 +7519,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PB-047</t>
+          <t>PB-052</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Start 1</t>
+          <t>Pause 1</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>LxStart 0</t>
+          <t>LxPause 0</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -7496,9 +7538,13 @@
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>V2.89 + real LCR: Pause with no delivery open is accepted (rc 0, devSt 0x21 in the golden capture); the tracker's LxPause 1 is the V3.01 firmware guard</t>
+        </is>
+      </c>
       <c r="H87" t="n">
-        <v>835</v>
+        <v>569.8</v>
       </c>
     </row>
     <row r="88">
@@ -7507,17 +7553,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PB-084</t>
+          <t>PB-047</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>GetLastMtrCmd 1</t>
+          <t>Start 1</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>LxGetLastMtrCmd 1,Start,0</t>
+          <t>LxStart 0</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -7528,7 +7574,7 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>541.9</v>
+        <v>571.3</v>
       </c>
     </row>
     <row r="89">
@@ -7537,17 +7583,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PB-075</t>
+          <t>PB-084</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SwitchState 1</t>
+          <t>GetLastMtrCmd 1</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>LxSwitchState 1,Run</t>
+          <t>LxGetLastMtrCmd 1,Start,0</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -7556,13 +7602,9 @@
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>delivery open</t>
-        </is>
-      </c>
+      <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>534.6</v>
+        <v>607.6</v>
       </c>
     </row>
     <row r="90">
@@ -7571,17 +7613,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PB-012</t>
+          <t>PB-075</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>SwitchState 2</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,254,1790376049,5.6,60.0,5159.3,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxSwitchState 1,Run</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -7592,8 +7634,11 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>flowing after Start</t>
-        </is>
+          <t>delivery open</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>540.3</v>
       </c>
     </row>
     <row r="91">
@@ -7602,7 +7647,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PB-099</t>
+          <t>PB-012</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -7612,7 +7657,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,0,1790376051,7.6,60.0,5161.3,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxGetData 1,1,132,1790405499,5.7,60.0,5396.5,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -7623,7 +7668,7 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>gross and totalizer rising</t>
+          <t>flowing after Start</t>
         </is>
       </c>
     </row>
@@ -7638,12 +7683,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>GetData 1 0 x2</t>
+          <t>GetData 1 0</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,254,1790376049,5.6,60.0,5159.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetData 1,1,0,1790376051,7.6,60.0,5161.3,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxGetData 1,1,134,1790405501,7.7,60.0,5398.6,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -7654,7 +7699,7 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>volume accrues</t>
+          <t>gross and totalizer rising</t>
         </is>
       </c>
     </row>
@@ -7664,17 +7709,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PB-051</t>
+          <t>PB-099</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Pause 1</t>
+          <t>GetData 1 0 x2</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>LxPause 0</t>
+          <t>LxGetData 1,1,132,1790405499,5.7,60.0,5396.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetData 1,1,134,1790405501,7.7,60.0,5398.6,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -7683,9 +7728,10 @@
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="n">
-        <v>577.9</v>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>volume accrues</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -7699,12 +7745,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>Pause 1</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,4,1790376055,9.1,0.0,5162.7,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxPause 0</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -7713,10 +7759,9 @@
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>paused: flow 0</t>
-        </is>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="n">
+        <v>564.1</v>
       </c>
     </row>
     <row r="95">
@@ -7725,17 +7770,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PB-101</t>
+          <t>PB-051</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>GetData 1 0 (paused)</t>
+          <t>GetData 1 0</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,6,1790376057,9.1,0.0,5162.7,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxGetData 1,1,138,1790405505,9.1,0.0,5399.9,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -7746,7 +7791,7 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>no volume while paused</t>
+          <t>paused: flow 0</t>
         </is>
       </c>
     </row>
@@ -7756,17 +7801,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PB-047</t>
+          <t>PB-101</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Start 1</t>
+          <t>GetData 1 0 (paused)</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>LxStart 0</t>
+          <t>LxGetData 1,1,140,1790405507,9.1,0.0,5399.9,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -7777,11 +7822,8 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>resume</t>
-        </is>
-      </c>
-      <c r="H96" t="n">
-        <v>766.2</v>
+          <t>no volume while paused</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -7795,12 +7837,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>Start 1</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,10,1790376061,11.7,60.0,5165.4,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxStart 0</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -7811,8 +7853,11 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>flowing again after resume</t>
-        </is>
+          <t>resume</t>
+        </is>
+      </c>
+      <c r="H97" t="n">
+        <v>568.2</v>
       </c>
     </row>
     <row r="98">
@@ -7821,17 +7866,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PB-054</t>
+          <t>PB-047</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Stop 1</t>
+          <t>GetData 1 0</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>LxStop 0</t>
+          <t>LxGetData 1,1,145,1790405512,12.7,60.0,5403.5,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -7840,9 +7885,10 @@
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="n">
-        <v>570.7</v>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>flowing again after resume</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -7856,12 +7902,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>Stop 1</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,14,1790376065,13.2,0.0,5166.9,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxStop 0</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -7870,10 +7916,9 @@
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>stopped: flow 0</t>
-        </is>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="n">
+        <v>569</v>
       </c>
     </row>
     <row r="100">
@@ -7887,12 +7932,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>GetData 1 0 (final)</t>
+          <t>GetData 1 0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,14,1790376065,13.2,0.0,5166.9,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxGetData 1,1,148,1790405515,13.4,0.0,5404.2,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -7903,7 +7948,7 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>ticket math</t>
+          <t>stopped: flow 0</t>
         </is>
       </c>
     </row>
@@ -7913,17 +7958,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PB-084</t>
+          <t>PB-054</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>GetLastMtrCmd 1</t>
+          <t>GetData 1 0 (final)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>LxGetLastMtrCmd 1,Stop,0</t>
+          <t>LxGetData 1,1,148,1790405515,13.4,0.0,5404.2,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -7932,9 +7977,10 @@
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="n">
-        <v>774.8</v>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>ticket math</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -7943,17 +7989,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PB-048</t>
+          <t>PB-084</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Start 99</t>
+          <t>GetLastMtrCmd 1</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>LxStart 1</t>
+          <t>LxGetLastMtrCmd 1,Stop,0</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -7964,7 +8010,7 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>534.7</v>
+        <v>539.8</v>
       </c>
     </row>
     <row r="103">
@@ -7973,17 +8019,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PB-053</t>
+          <t>PB-048</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Pause 99</t>
+          <t>Start 99</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>LxPause 1</t>
+          <t>LxStart 1</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -7994,7 +8040,7 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>547.3</v>
+        <v>538.4</v>
       </c>
     </row>
     <row r="104">
@@ -8003,17 +8049,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PB-056</t>
+          <t>PB-053</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Stop 99</t>
+          <t>Pause 99</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>LxStop 1</t>
+          <t>LxPause 1</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -8024,7 +8070,7 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>640.7</v>
+        <v>536.9</v>
       </c>
     </row>
     <row r="105">
@@ -8033,17 +8079,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PB-004</t>
+          <t>PB-056</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>HisDataTime 1</t>
+          <t>Stop 99</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>LxHisDataTime 1,1790376044,1790376063,</t>
+          <t>LxStop 1</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -8054,7 +8100,7 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>534.8</v>
+        <v>546.9</v>
       </c>
     </row>
     <row r="106">
@@ -8063,17 +8109,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PB-007</t>
+          <t>PB-004</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>BoxStorage 1</t>
+          <t>HisDataTime 1</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>LxBoxStorage 1,15,24640,</t>
+          <t>LxHisDataTime 1,1790405494,1790405513,</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -8081,14 +8127,10 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>records expected</t>
-        </is>
-      </c>
+      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>542.2</v>
+        <v>712.8</v>
       </c>
     </row>
     <row r="107">
@@ -8097,17 +8139,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PB-010</t>
+          <t>PB-007</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>GetData 1,1</t>
+          <t>BoxStorage 1</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>LxGetDataTs 1,0,1,1790376044,0.7,60.0,5154.3,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxBoxStorage 1,15,24640,</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -8115,10 +8157,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>records expected</t>
+        </is>
+      </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>904.1</v>
+        <v>541.6</v>
       </c>
     </row>
     <row r="108">
@@ -8132,12 +8178,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>GetDataEcho 1,0,1</t>
+          <t>GetData 1,1</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>LxGetDataTs 1,0,2,1790376045,1.7,60.0,5155.3,0.0,5153.6,0.0,0.0,S,0.0,E</t>
+          <t>LxGetDataTs 1,0,6,1790405494,0.7,60.0,5391.6,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -8146,13 +8192,9 @@
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>ack -&gt; next record</t>
-        </is>
-      </c>
+      <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>750.6</v>
+        <v>543</v>
       </c>
     </row>
     <row r="109">
@@ -8161,17 +8203,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PB-016</t>
+          <t>PB-010</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>GetDataTs 1,1790376040,1790376077</t>
+          <t>GetDataEcho 6,0,1</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>LxGetDataTs 1,1,1790376045,1.7,60.0,5155.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,2,1790376046,2.6,60.0,5156.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,3,1790376047,3.6,60.0,5157.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,4,1790376048,4.6,60.0,5158.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,5,1790376049,5.6,60.0,5159.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,6,1790376050,6.6,60.0,5160.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,7,1790376051,7.6,60.0,5161.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,8,1790376052,8.7,60.0,5162.3,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,9,1790376053,9.1,0.0,5162.7,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,10,1790376059,9.7,60.0,5163.4,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,11,1790376060,10.7,60.0,5164.4,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,12,1790376061,11.7,60.0,5165.4,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,13,1790376062,12.7,60.0,5166.4,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,14,1790376063,13.2,0.0,5166.9,0.0,5153.6,0.0,0.0,S,0.0,E | LxGetDataTs 1,</t>
+          <t>LxGetDataTs 1,0,7,1790405495,1.7,60.0,5392.5,0.0,5390.8,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -8179,18 +8221,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>records in range expected</t>
-        </is>
-      </c>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>tracker range 1700000000.. is before this box's clock; using the delivery window</t>
+          <t>ack -&gt; next record</t>
         </is>
       </c>
       <c r="H109" t="n">
-        <v>662.4</v>
+        <v>548.8</v>
       </c>
     </row>
     <row r="110">
@@ -8199,17 +8237,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PB-108</t>
+          <t>PB-016</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>PresetGross 1,5.0</t>
+          <t>GetDataTs 1,1790405490,1790405526</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>LxPresetGross 0</t>
+          <t>LxGetDataTs 1,1,1790405495,1.7,60.0,5392.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,2,1790405496,2.7,60.0,5393.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,3,1790405497,3.7,60.0,5394.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,4,1790405498,4.7,60.0,5395.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,5,1790405499,5.7,60.0,5396.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,6,1790405500,6.7,60.0,5397.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,7,1790405501,7.7,60.0,5398.6,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,8,1790405502,8.7,60.0,5399.6,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,9,1790405503,9.1,0.0,5399.9,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,10,1790405509,9.6,60.0,5400.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,11,1790405510,10.6,60.0,5401.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,12,1790405511,11.6,60.0,5402.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,13,1790405512,12.7,60.0,5403.5,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,14,1790405513,13.4,0.0,5404.2,0.0,5390.8,0.0,0.0,S,0.0,E | LxGetDataTs 1,</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -8217,10 +8255,18 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>records in range expected</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>tracker range 1700000000.. is before this box's clock; using the delivery window</t>
+        </is>
+      </c>
       <c r="H110" t="n">
-        <v>585.3</v>
+        <v>674.5</v>
       </c>
     </row>
     <row r="111">
@@ -8234,12 +8280,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Start 1</t>
+          <t>PresetGross 1,5.0</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>LxStart 0</t>
+          <t>LxPresetGross 0</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -8250,7 +8296,7 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>775.2</v>
+        <v>584.7</v>
       </c>
     </row>
     <row r="112">
@@ -8264,12 +8310,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>Start 1</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,31,1790376082,5.0,0.0,5171.9,0.0,5166.9,0.0,0.0,S,0.0,E</t>
+          <t>LxStart 0</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -8278,10 +8324,9 @@
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>preset reached</t>
-        </is>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="n">
+        <v>714.4</v>
       </c>
     </row>
     <row r="113">
@@ -8290,17 +8335,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SETUP</t>
+          <t>PB-108</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Stop 1</t>
+          <t>GetData 1 0</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>LxStop 0</t>
+          <t>LxGetData 1,1,165,1790405532,5.0,0.0,5409.2,0.0,5404.2,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -8309,9 +8354,10 @@
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="n">
-        <v>571.8</v>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>preset reached</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -8325,12 +8371,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>PresetGross 1,0</t>
+          <t>Stop 1</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>LxPresetGross 0</t>
+          <t>LxStop 0</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -8341,7 +8387,7 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>874</v>
+        <v>577.9</v>
       </c>
     </row>
     <row r="115">
@@ -8350,17 +8396,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PB-095</t>
+          <t>SETUP</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Start 1</t>
+          <t>PresetGross 1,0</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>LxStart 0</t>
+          <t>LxPresetGross 0</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -8371,7 +8417,7 @@
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>765.2</v>
+        <v>586</v>
       </c>
     </row>
     <row r="116">
@@ -8380,12 +8426,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PB-095</t>
+          <t>PB-106</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Start 2</t>
+          <t>Start 1</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -8401,7 +8447,7 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>563.5</v>
+        <v>571.2</v>
       </c>
     </row>
     <row r="117">
@@ -8410,17 +8456,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PB-095</t>
+          <t>PB-106</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>RdRegister</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,39,1790376090,4.6,60.0,5176.6,0.0,5171.9,0.0,0.0,S,0.0,E</t>
+          <t>LxRdRegister 0,0</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -8431,8 +8477,11 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>meter 1 flowing</t>
-        </is>
+          <t>meter offline</t>
+        </is>
+      </c>
+      <c r="H117" t="n">
+        <v>598.4</v>
       </c>
     </row>
     <row r="118">
@@ -8441,17 +8490,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PB-095</t>
+          <t>PB-106</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>GetData 2 0</t>
+          <t>GetData 1 0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>LxGetData 2,1,36,1790376091,3.3,45.0,49295.4,0.0,49292.0,0.0,0.0,S,0.0,E</t>
+          <t>LxGetData Error,</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -8462,8 +8511,11 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>meter 2 flowing (independent)</t>
-        </is>
+          <t>no live data from an offline meter</t>
+        </is>
+      </c>
+      <c r="H118" t="n">
+        <v>538.9</v>
       </c>
     </row>
     <row r="119">
@@ -8472,7 +8524,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>PB-095</t>
+          <t>PB-106</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -8482,7 +8534,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>LxStop 0</t>
+          <t>LxStop 1</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -8491,9 +8543,13 @@
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>command not delivered</t>
+        </is>
+      </c>
       <c r="H119" t="n">
-        <v>786.8</v>
+        <v>1035.8</v>
       </c>
     </row>
     <row r="120">
@@ -8502,17 +8558,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PB-095</t>
+          <t>PB-106</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Stop 2</t>
+          <t>BoxStatus</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>LxStop 0</t>
+          <t>LxBoxStatus 2,0,0,1,0.0,S,0.0,E,0,1</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -8521,9 +8577,13 @@
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>box still answers the app</t>
+        </is>
+      </c>
       <c r="H120" t="n">
-        <v>565.6</v>
+        <v>540.9</v>
       </c>
     </row>
     <row r="121">
@@ -8532,17 +8592,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PB-095</t>
+          <t>PB-106</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>RdRegister</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,44,1790376095,7.0,0.0,5178.9,0.0,5171.9,0.0,0.0,S,0.0,E</t>
+          <t>LxRdRegister 0,1</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -8553,8 +8613,11 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>meter 1 stopped</t>
-        </is>
+          <t>meter back online after reconnect</t>
+        </is>
+      </c>
+      <c r="H121" t="n">
+        <v>600.5</v>
       </c>
     </row>
     <row r="122">
@@ -8563,17 +8626,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>PB-095</t>
+          <t>PB-106</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>GetData 2 0</t>
+          <t>GetData 1 0</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>LxGetData 2,1,41,1790376096,4.6,0.0,49296.6,0.0,49292.0,0.0,0.0,S,0.0,E</t>
+          <t>LxGetData 1,1,173,1790405548,13.5,60.0,5422.7,0.0,5409.2,0.0,0.0,S,0.0,E</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -8584,7 +8647,7 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>meter 2 stopped</t>
+          <t>delivery kept running on the meter while unplugged</t>
         </is>
       </c>
     </row>
@@ -8594,17 +8657,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>PB-007</t>
+          <t>PB-106</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>BoxStorage 2</t>
+          <t>Stop 1</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>LxBoxStorage 2,8,25088,</t>
+          <t>LxStop 0</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -8612,14 +8675,10 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>records expected</t>
-        </is>
-      </c>
+      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>540.5</v>
+        <v>584.8</v>
       </c>
     </row>
     <row r="124">
@@ -8628,17 +8687,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>PB-106</t>
+          <t>PB-023</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Start 1</t>
+          <t>SetBtName PandaBox1</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>LxStart 0</t>
+          <t>LxSetBtName 0</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -8649,7 +8708,7 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>564.5</v>
+        <v>610.3</v>
       </c>
     </row>
     <row r="125">
@@ -8658,17 +8717,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>PB-106</t>
+          <t>PB-023</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>RdRegister</t>
+          <t>RdBtName</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>LxRdRegister 0,0</t>
+          <t>LxRdBtName PandaBox1</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -8677,13 +8736,9 @@
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>both meters offline</t>
-        </is>
-      </c>
+      <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>597.8</v>
+        <v>539.2</v>
       </c>
     </row>
     <row r="126">
@@ -8692,17 +8747,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>PB-106</t>
+          <t>SETUP</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>SetBtName PandaBrain</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>LxGetData Error,</t>
+          <t>LxSetBtName 0</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -8711,13 +8766,9 @@
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>no live data from an offline meter</t>
-        </is>
-      </c>
+      <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>539.4</v>
+        <v>548.3</v>
       </c>
     </row>
     <row r="127">
@@ -8726,17 +8777,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>PB-106</t>
+          <t>PB-041</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Stop 1</t>
+          <t>BoxReset</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>LxStop 1</t>
+          <t>LxBoxReset 0</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -8745,13 +8796,9 @@
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>command not delivered</t>
-        </is>
-      </c>
+      <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>1240.9</v>
+        <v>536.7</v>
       </c>
     </row>
     <row r="128">
@@ -8760,19 +8807,15 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>PB-106</t>
+          <t>PB-041</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>BoxStatus</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>LxBoxStatus 2,0,1,2,0.0,S,0.0,E,0,1</t>
-        </is>
-      </c>
+          <t>reconnect after BoxReset</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -8781,11 +8824,8 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>box still answers the app</t>
-        </is>
-      </c>
-      <c r="H128" t="n">
-        <v>541.9</v>
+          <t>box rebooted and advertises again</t>
+        </is>
       </c>
     </row>
     <row r="129">
@@ -8794,17 +8834,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>PB-106</t>
+          <t>PB-041</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>RdRegister</t>
+          <t>BoxInfo</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>LxRdRegister 1,1</t>
+          <t>LxBoxInfo 2.4,250502,2.901,260925,860858062040217,LCR</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -8813,13 +8853,9 @@
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>meters back online after reconnect</t>
-        </is>
-      </c>
+      <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>827</v>
+        <v>803.7</v>
       </c>
     </row>
     <row r="130">
@@ -8828,17 +8864,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PB-106</t>
+          <t>PB-041</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>GetData 1 0</t>
+          <t>SetBoxTime 1790405610</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>LxGetData 1,1,52,1790376111,13.5,60.0,5192.5,0.0,5178.9,0.0,0.0,S,0.0,E</t>
+          <t>LxSetBoxTime 0</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -8847,247 +8883,9 @@
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>delivery kept running on the meter while unplugged</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="n">
-        <v>130</v>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>PB-106</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>Stop 1</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>LxStop 0</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="n">
-        <v>577.4</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="n">
-        <v>131</v>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>PB-023</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>SetBtName PandaBox1</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>LxSetBtName 0</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="n">
-        <v>611.2</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="n">
-        <v>132</v>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>PB-023</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>RdBtName</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>LxRdBtName PandaBox1</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr"/>
-      <c r="G133" t="inlineStr"/>
-      <c r="H133" t="n">
-        <v>536.8</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="n">
-        <v>133</v>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>SETUP</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>SetBtName PandaBrain</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>LxSetBtName 0</t>
-        </is>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F134" t="inlineStr"/>
-      <c r="G134" t="inlineStr"/>
-      <c r="H134" t="n">
-        <v>541.9</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="n">
-        <v>134</v>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>PB-041</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>BoxReset</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>LxBoxReset 0</t>
-        </is>
-      </c>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F135" t="inlineStr"/>
-      <c r="G135" t="inlineStr"/>
-      <c r="H135" t="n">
-        <v>535.3</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="n">
-        <v>135</v>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>PB-041</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>reconnect after BoxReset</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr"/>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>box rebooted and advertises again</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="n">
-        <v>136</v>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>PB-041</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>BoxInfo</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>LxBoxInfo 2.4,250502,2.901,260925,860858062040217,LCR</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr"/>
-      <c r="H137" t="n">
-        <v>623.1</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="n">
-        <v>137</v>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>PB-041</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>SetBoxTime 1790376197</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>LxSetBoxTime 0</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr"/>
-      <c r="H138" t="n">
-        <v>541</v>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="n">
+        <v>547.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>